<commit_message>
Commit week 5 6 7
</commit_message>
<xml_diff>
--- a/DE190592_NguyenThanhNhan_AIAuditlog.xlsx
+++ b/DE190592_NguyenThanhNhan_AIAuditlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhannguyenthanh/FPT/Kì 5/SWP391/AI_AuditLog/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83F12168-1EE6-0B48-80C0-48088B5395D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC104CFB-AF89-FF4C-AB12-06B37B82B835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="36040" yWindow="1180" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="316">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -707,6 +707,352 @@
   </si>
   <si>
     <t>System architecture diagram + module list</t>
+  </si>
+  <si>
+    <t>Business Rules</t>
+  </si>
+  <si>
+    <t>Cần định nghĩa các quy tắc ràng buộc rõ ràng khi bệnh nhân đặt lịch hẹn tái khám da liễu định kỳ.</t>
+  </si>
+  <si>
+    <t>What business rules should be applied to scheduling follow-up dermatology appointments?</t>
+  </si>
+  <si>
+    <t>AI suggested rules for minimum interval between visits, doctor availability sync, and auto-cancellation for no-shows.</t>
+  </si>
+  <si>
+    <t>Appointment Business Rules Document</t>
+  </si>
+  <si>
+    <t>Treatment Plan AI</t>
+  </si>
+  <si>
+    <t>Làm thế nào để AI gợi ý phác đồ điều trị tự động dựa trên kết quả phân tích loại da và mức độ tổn thương.</t>
+  </si>
+  <si>
+    <t>How can AI generate personalized dermatology treatment plans based on skin analysis outputs?</t>
+  </si>
+  <si>
+    <t>AI proposed using a knowledge graph combined with LLMs to map skin severity scores to clinical guidelines and product recommendations.</t>
+  </si>
+  <si>
+    <t>Treatment Generation Architecture + Prompt Flow</t>
+  </si>
+  <si>
+    <t>Chatbot Integration</t>
+  </si>
+  <si>
+    <t>Kiểm tra tính chính xác và giới hạn phạm vi tư vấn của Chatbot qua API để tránh tư vấn sai chuyên môn y tế.</t>
+  </si>
+  <si>
+    <t>How can we test and set guardrails for a dermatology consultation chatbot via API?</t>
+  </si>
+  <si>
+    <t>AI suggested prompt engineering guardrails, intent classification, and a strict fallback mechanism when queries touch critical medical diagnostics.</t>
+  </si>
+  <si>
+    <t>Chatbot Guardrails Specification + Test Cases</t>
+  </si>
+  <si>
+    <t>Requirement Optimization</t>
+  </si>
+  <si>
+    <t>Tối ưu hóa các yêu cầu phần mềm bị mơ hồ (ambiguous requirements) trong hồ sơ bệnh án điện tử để tổ phát triển dễ triển khai.</t>
+  </si>
+  <si>
+    <t>How can we use AI to detect and resolve ambiguous software requirements in electronic medical records (EMR)?</t>
+  </si>
+  <si>
+    <t>AI suggested utilizing NLP techniques to parse requirements, highlighting vague terms like "fast loading" or "flexible data entry".</t>
+  </si>
+  <si>
+    <t>Optimized SRS Document + Ambiguity Report</t>
+  </si>
+  <si>
+    <t>Screen Specification</t>
+  </si>
+  <si>
+    <t>Định nghĩa các trường thông tin và bố cục chi tiết cho màn hình "Kết Quả Soi Da" của Bệnh nhân.</t>
+  </si>
+  <si>
+    <t>What are the essential UI components and fields for a patient's Skin Analysis Result screen?</t>
+  </si>
+  <si>
+    <t>AI recommended including visual severity charts, before/after comparisons, AI score highlights, and doctor's notes section.</t>
+  </si>
+  <si>
+    <t>Patient Screen Wireframe + Component Specs</t>
+  </si>
+  <si>
+    <t>API Performance</t>
+  </si>
+  <si>
+    <t>Kiểm tra hiệu năng phản hồi của API phân tích hình ảnh da mặt khi có nhiều bác sĩ cùng sử dụng một lúc.</t>
+  </si>
+  <si>
+    <t>How should we load test the AI skin analysis API endpoints in a clinic management system?</t>
+  </si>
+  <si>
+    <t>AI suggested using JMeter or Artillery to simulate concurrent image upload requests and monitor response latency.</t>
+  </si>
+  <si>
+    <t>Performance Test Report (JMeter)</t>
+  </si>
+  <si>
+    <t>Report &amp; Analytics</t>
+  </si>
+  <si>
+    <t>Cần thiết kế phân hệ báo cáo để thống kê doanh thu và tần suất các nhóm bệnh da liễu phổ biến tại phòng khám.</t>
+  </si>
+  <si>
+    <t>What metrics and visualization types should be included in a dermatology clinic analytics dashboard?</t>
+  </si>
+  <si>
+    <t>AI suggested charts for revenue by service, patient demographics, medication consumption, and top skin conditions treated.</t>
+  </si>
+  <si>
+    <t>Dashboard Mockup + Analytics Schema</t>
+  </si>
+  <si>
+    <t>Notification System</t>
+  </si>
+  <si>
+    <t>Xử lý việc tự động gửi thông báo nhắc lịch chăm sóc da và uống thuốc định kỳ cho bệnh nhân theo phác đồ.</t>
+  </si>
+  <si>
+    <t>How to design an automated notification system for skincare routines and medication reminders?</t>
+  </si>
+  <si>
+    <t>AI proposed a cron-job architecture combined with Firebase Cloud Messaging (FCM) or Twilio for SMS/Push notifications.</t>
+  </si>
+  <si>
+    <t>Notification Workflow + Database Triggers</t>
+  </si>
+  <si>
+    <t>Data Privacy</t>
+  </si>
+  <si>
+    <t>Đảm bảo tính bảo mật và quyền riêng tư đối với hình ảnh khuôn mặt tổn thương của bệnh nhân.</t>
+  </si>
+  <si>
+    <t>What compliance and security measures are needed for storing patient facial images in a clinic system?</t>
+  </si>
+  <si>
+    <t>AI recommended data encryption at rest (AES-256), secure AWS S3 buckets, and access token validation for image URLs.</t>
+  </si>
+  <si>
+    <t>Security Architecture Document</t>
+  </si>
+  <si>
+    <t>Telehealth Integration</t>
+  </si>
+  <si>
+    <t>Tích hợp tính năng tư vấn từ xa (Telehealth) cho các trường hợp bệnh nhân muốn tái khám online.</t>
+  </si>
+  <si>
+    <t>How can video-consultation (Telehealth) capabilities be integrated into DermaSmart?</t>
+  </si>
+  <si>
+    <t>AI suggested integrating WebRTC or third-party APIs like Zoom/Agora for video calls, paired with chat messaging.</t>
+  </si>
+  <si>
+    <t>Telehealth Architecture &amp; UI Mockup</t>
+  </si>
+  <si>
+    <t>Medical Record Versioning</t>
+  </si>
+  <si>
+    <t>Xử lý việc cập nhật và lưu vết lịch sử (audit trail) mỗi khi bác sĩ thay đổi thông tin bệnh án của bệnh nhân.</t>
+  </si>
+  <si>
+    <t>How should we implement history tracking (audit log) for electronic medical records in SQL Server?</t>
+  </si>
+  <si>
+    <t>Database Audit Log Schema</t>
+  </si>
+  <si>
+    <t>Testing Strategy</t>
+  </si>
+  <si>
+    <t>Xây dựng kịch bản kiểm thử (Test Cases) đảm bảo tính chính xác của chức năng trừ kho tự động khi xuất dược mỹ phẩm.</t>
+  </si>
+  <si>
+    <t>Create a comprehensive test plan for the automated inventory deduction feature in DermaSmart.</t>
+  </si>
+  <si>
+    <t>AI provided test scenarios including normal checkout, stockouts, simultaneous purchasing, and order cancellation reversals.</t>
+  </si>
+  <si>
+    <t>Inventory Test Cases Document</t>
+  </si>
+  <si>
+    <t>Role-Based Access</t>
+  </si>
+  <si>
+    <t>Kiểm thử ma trận phân quyền (RBAC) để đảm bảo nhân viên lễ tân không thể xem chi tiết bệnh lý nhạy cảm của khách hàng.</t>
+  </si>
+  <si>
+    <t>How to verify that Role-Based Access Control (RBAC) strictly prevents unauthorized roles from accessing EMR details?</t>
+  </si>
+  <si>
+    <t>AI suggested writing Integration tests using different role tokens to assert that endpoints return 403 Forbidden for restricted roles.</t>
+  </si>
+  <si>
+    <t>Security Test Report + RBAC Verification</t>
+  </si>
+  <si>
+    <t>Feedback System</t>
+  </si>
+  <si>
+    <t>Xây dựng chức năng đánh giá dịch vụ và thu thập phản hồi của bệnh nhân sau mỗi liệu trình điều trị da liễu.</t>
+  </si>
+  <si>
+    <t>What is the best design for a patient satisfaction feedback and review system in a clinic application?</t>
+  </si>
+  <si>
+    <t>AI suggested implementing a 5-star rating system combined with structured tags (e.g., "Friendly staff", "Clean clinic") and open text.</t>
+  </si>
+  <si>
+    <t>Feedback Module UI Wireframe + Database Schema</t>
+  </si>
+  <si>
+    <t>Database Scaling</t>
+  </si>
+  <si>
+    <t>Thiết kế cấu trúc lưu trữ cơ sở dữ liệu để tối ưu cho việc truy vấn lịch sử điều trị kéo dài nhiều năm của bệnh nhân.</t>
+  </si>
+  <si>
+    <t>How to optimize database indexing for fast retrieval of historical patient medical records?</t>
+  </si>
+  <si>
+    <t>Database Indexing Plan</t>
+  </si>
+  <si>
+    <t>Chatbot Fallback</t>
+  </si>
+  <si>
+    <t>Xử lý trường hợp Chatbot không hiểu câu hỏi phức tạp hoặc gặp câu hỏi mang tính khẩn cấp về y tế (Fallback Mechanism).</t>
+  </si>
+  <si>
+    <t>What fallback strategies should a medical chatbot use when it cannot confidently answer a user's query?</t>
+  </si>
+  <si>
+    <t>AI suggested routing the conversation to a human receptionist, offering a list of hotlines, or providing standard clarification prompts.</t>
+  </si>
+  <si>
+    <t>Chatbot Fallback Flow Diagram</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Quy tắc đặt lịch phải linh hoạt theo từng loại bệnh án.Contextualization: Bệnh nhân mụn trứng cá cần tái khám sau 2-4 tuần, còn treatment nặng cần theo dõi sát hơn.Creative Synthesis: Kết hợp trạng thái hồ sơ bệnh án để tự động gợi ý khung giờ phù hợp.Decision: Áp dụng bộ quy tắc Business Rules vào Module đặt lịch.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI chỉ đóng vai trò dự thảo phác đồ thô để tránh rủi ro pháp lý y khoa.Contextualization: Phác đồ cần phân tách rõ giữa thuốc kê đơn (Prescription) và dược mỹ phẩm dưỡng da (Skincare).Creative Synthesis: Thiết kế giao diện cho phép bác sĩ chỉnh sửa trực tiếp trên gợi ý của AI.Decision: Phát triển module AI Treatment Suggester dạng API nội bộ.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Chatbot không được phép đưa ra chẩn đoán bệnh thay bác sĩ.Contextualization: Chỉ tập trung tư vấn quy trình dịch vụ, đặt lịch và hướng dẫn sử dụng dược mỹ phẩm chăm sóc da.Creative Synthesis: Xây dựng bộ dữ liệu chặn (Blacklist keywords) các câu hỏi nguy hiểm.Decision: Triển khai Chatbot qua API với kịch bản kiểm thử nghiêm ngặt dựa trên Intent Testing.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Việc làm rõ yêu cầu giúp các thành viên (Nhân, Bảo, Thuận) đồng bộ nhanh hơn.Contextualization: Đồ án SWP391 cần tài liệu SRS cực kỳ tường minh để chấm điểm.Creative Synthesis: Sử dụng AI để viết lại các câu mơ hồ thành dạng cấu trúc Given-When-Then.Decision: Ứng dụng AI tối ưu hóa tài liệu đặc tả yêu cầu của hệ thống.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Giao diện phía bệnh nhân phải trực quan, dễ hiểu, tránh các thuật ngữ y khoa quá hàn lâm.Contextualization: Phù hợp với hiển thị trên cả thiết bị di động khi bệnh nhân tra cứu tại nhà.Creative Synthesis: Thêm thanh tiến trình (Progress Tracker) để thể hiện sự cải thiện của làn da qua các lần khám.Decision: Chốt bản thiết kế wireframe chi tiết cho màn hình Skin Result.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Thời gian phản hồi chậm sẽ làm gián đoạn quy trình khám trực tiếp của bác sĩ.Contextualization: Giới hạn tối đa là dưới 3 giây cho một lượt phân tích ảnh.Creative Synthesis: Áp dụng cơ chế hàng đợi (Queue) và nén ảnh tự động trước khi gửi lên AI model.Decision: Thực hiện Load testing và tối ưu cấu hình API Gateway.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Báo cáo phải giúp chủ phòng khám đưa ra quyết định nhập hàng dược mỹ phẩm chính xác.Contextualization: Dữ liệu cần được bảo mật và chỉ phân quyền cho Admin/Clinic Manager xem.Creative Synthesis: Tích hợp bộ lọc động theo mùa (vì bệnh da liễu thay đổi rất lớn giữa mùa đông và mùa hè).Decision: Xây dựng Module Analytics sử dụng Chart.js trên nền React.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Tần suất thông báo quá dày đặc có thể gây phiền (spam) cho bệnh nhân.Contextualization: Cho phép bệnh nhân chủ động bật/tắt hoặc hẹn giờ nhận thông báo trên app.Creative Synthesis: Nhắc lịch uống thuốc kèm theo hình ảnh nhận diện viên thuốc để tránh uống nhầm.Decision: Sử dụng Firebase Cloud Messaging để tối ưu chi phí và trải nghiệm cho đồ án.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Hình ảnh bệnh lý da mặt là dữ liệu nhạy cảm cao, rò rỉ sẽ ảnh hưởng nghiêm trọng đến phòng khám.Contextualization: Đảm bảo tuân thủ cơ bản các nguyên tắc an toàn dữ liệu y tế trong đồ án SWP391.Creative Synthesis: Che mờ (blur) vùng mắt tự động đối với các ảnh minh họa không cần thiết phải lộ toàn mặt.Decision: Triển khai cơ chế Pre-signed URL cho việc truy xuất hình ảnh từ S3.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Khám da liễu online đòi hỏi camera chất lượng cao; cần có cảnh báo giới hạn cho bệnh nhân trước khi vào cuộc gọi.Contextualization: Giúp tối ưu hóa thời gian trống của bác sĩ tại phòng khám.Creative Synthesis: Cho phép bác sĩ vừa gọi video vừa mở song song hồ sơ bệnh án và ảnh soi da trên cùng một màn hình.Decision: Lựa chọn giải pháp WebRTC đơn giản để tự phát triển nhằm tối ưu hóa điểm kỹ thuật đồ án.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Bệnh án y khoa là căn cứ pháp lý, mọi chỉnh sửa bắt buộc phải lưu lại vết ai sửa, sửa lúc nào và sửa cái gì.Contextualization: Hệ thống cần truy xuất lịch sử chỉnh sửa này một cách nhanh chóng khi có tranh chấp.Creative Synthesis: Thiết kế giao diện so sánh các phiên bản bệnh án cũ - mới theo dạng diff-view trực quan.Decision: Tạo bảng EMR_History để lưu trữ dữ liệu dưới dạng JSON các thay đổi.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Lỗi trừ sai kho sẽ dẫn đến mất mát tài chính và sai lệch số liệu kế toán phòng khám.Contextualization: Cần test kỹ trường hợp bất đồng bộ (concurrency) khi hai nhân viên cùng xuất một mặt hàng cuối cùng.Creative Synthesis: Áp dụng kỹ thuật Lock trong Database để xử lý tranh chấp dữ liệu kho.Decision: Thực hiện viết Unit Test và Integration Test tự động cho Module Inventory.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Phân quyền không chặt chẽ là lỗi bảo mật nghiêm trọng trong đánh giá đồ án phần mềm.Contextualization: Nhân viên tiếp tân chỉ được xem thông tin hành chính và trạng thái thanh toán, không được xem chi tiết bệnh án.Creative Synthesis: Xây dựng Middleware phân quyền tập trung ở Backend để quản lý tất cả API endpoints.Decision: Sử dụng Spring Security để hiện thực hóa cấu trúc phân quyền RBAC chặt chẽ.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Phản hồi của khách hàng giúp nâng cao chất lượng dịch vụ của phòng khám.Contextualization: Hệ thống sẽ tự động gửi link đánh giá qua thông báo app sau khi bệnh nhân hoàn thành bước "Thanh toán &amp; Nhận thuốc".Creative Synthesis: Sử dụng AI để phân tích sắc thái cảm xúc (Sentiment Analysis) từ phản hồi văn bản để lọc ra các phàn nàn khẩn cấp.Decision: Triển khai Module Feedback cơ bản phục vụ báo cáo chất lượng cho Quản lý.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Truy vấn chậm khi tìm kiếm lịch sử y khoa sẽ làm tăng thời gian chờ đợi của bệnh nhân tại quầy.Contextualization: Dữ liệu lịch sử cần được tối ưu hóa bằng các chỉ mục (Indexes) phức hợp phù hợp.Creative Synthesis: Áp dụng kỹ thuật Lazy Loading trên giao diện để cDecision: Tạo Composite Index trên các trường khóa ngoại hay truy vấn của bảng bệnh án.hỉ tải dữ liệu các năm gần nhất trước.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Tránh để Chatbot trả lời sai lệch (hallucination) trong bối cảnh y tế vì có thể gây nguy hiểm.Contextualization: Nếu độ tự tin (Confidence Score) dưới 70%, Chatbot lập tức chuyển sang chế độ chuyển tiếp tin nhắn cho nhân viên.Creative Synthesis: Tạo nút bấm "Kết nối với tư vấn viên" hiển thị ngay lập tức khi Chatbot gặp bế tắc.Decision: Cấu hình ngưỡng tin cậy trên API Chatbot và thiết lập luồng chuyển đổi mượt mà sang nhân viên trực trực tiếp.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">AI suggested using Temporal Tables or creating a dedicated </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>AuditLog</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> table triggered on update/delete actions.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">AI recommended indexing on </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>PatientID</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>CreatedDate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>, and partitioning tables if historical data grows exponentially.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -716,7 +1062,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -792,6 +1138,31 @@
       <sz val="10"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -846,7 +1217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -901,6 +1272,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -917,8 +1291,26 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1233,14 +1625,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
     </row>
     <row r="3" spans="1:6" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1459,7 +1851,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:O57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1472,28 +1864,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
     </row>
     <row r="2" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:12" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
@@ -1882,9 +2274,9 @@
       <c r="H16" s="23" t="s">
         <v>201</v>
       </c>
-      <c r="I16" s="30"/>
-    </row>
-    <row r="17" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I16" s="24"/>
+    </row>
+    <row r="17" spans="1:15" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="23">
         <v>14</v>
       </c>
@@ -1909,9 +2301,9 @@
       <c r="H17" s="23" t="s">
         <v>207</v>
       </c>
-      <c r="I17" s="30"/>
-    </row>
-    <row r="18" spans="1:9" s="23" customFormat="1" ht="96" x14ac:dyDescent="0.2">
+      <c r="I17" s="24"/>
+    </row>
+    <row r="18" spans="1:15" s="23" customFormat="1" ht="96" x14ac:dyDescent="0.2">
       <c r="A18" s="23">
         <v>20</v>
       </c>
@@ -1937,7 +2329,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="19" spans="1:9" s="23" customFormat="1" ht="96" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15" s="23" customFormat="1" ht="96" x14ac:dyDescent="0.2">
       <c r="A19" s="23">
         <v>21</v>
       </c>
@@ -1962,6 +2354,908 @@
       <c r="H19" s="23" t="s">
         <v>219</v>
       </c>
+    </row>
+    <row r="20" spans="1:15" ht="96" x14ac:dyDescent="0.2">
+      <c r="A20" s="34">
+        <v>22</v>
+      </c>
+      <c r="B20" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="34" t="s">
+        <v>220</v>
+      </c>
+      <c r="D20" s="34" t="s">
+        <v>221</v>
+      </c>
+      <c r="E20" s="34" t="s">
+        <v>222</v>
+      </c>
+      <c r="F20" s="34" t="s">
+        <v>223</v>
+      </c>
+      <c r="G20" s="34" t="s">
+        <v>298</v>
+      </c>
+      <c r="H20" s="34" t="s">
+        <v>224</v>
+      </c>
+      <c r="I20" s="33"/>
+      <c r="J20" s="33"/>
+      <c r="K20" s="33"/>
+      <c r="L20" s="33"/>
+      <c r="M20" s="33"/>
+      <c r="N20" s="33"/>
+      <c r="O20" s="33"/>
+    </row>
+    <row r="21" spans="1:15" ht="96" x14ac:dyDescent="0.2">
+      <c r="A21" s="34">
+        <v>23</v>
+      </c>
+      <c r="B21" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" s="34" t="s">
+        <v>225</v>
+      </c>
+      <c r="D21" s="34" t="s">
+        <v>226</v>
+      </c>
+      <c r="E21" s="34" t="s">
+        <v>227</v>
+      </c>
+      <c r="F21" s="34" t="s">
+        <v>228</v>
+      </c>
+      <c r="G21" s="34" t="s">
+        <v>299</v>
+      </c>
+      <c r="H21" s="34" t="s">
+        <v>229</v>
+      </c>
+      <c r="I21" s="33"/>
+      <c r="J21" s="33"/>
+      <c r="K21" s="33"/>
+      <c r="L21" s="33"/>
+      <c r="M21" s="33"/>
+      <c r="N21" s="33"/>
+      <c r="O21" s="33"/>
+    </row>
+    <row r="22" spans="1:15" ht="112" x14ac:dyDescent="0.2">
+      <c r="A22" s="34">
+        <v>24</v>
+      </c>
+      <c r="B22" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="34" t="s">
+        <v>230</v>
+      </c>
+      <c r="D22" s="34" t="s">
+        <v>231</v>
+      </c>
+      <c r="E22" s="34" t="s">
+        <v>232</v>
+      </c>
+      <c r="F22" s="34" t="s">
+        <v>233</v>
+      </c>
+      <c r="G22" s="34" t="s">
+        <v>300</v>
+      </c>
+      <c r="H22" s="34" t="s">
+        <v>234</v>
+      </c>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="33"/>
+      <c r="N22" s="33"/>
+      <c r="O22" s="33"/>
+    </row>
+    <row r="23" spans="1:15" ht="96" x14ac:dyDescent="0.2">
+      <c r="A23" s="34">
+        <v>25</v>
+      </c>
+      <c r="B23" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="34" t="s">
+        <v>235</v>
+      </c>
+      <c r="D23" s="34" t="s">
+        <v>236</v>
+      </c>
+      <c r="E23" s="34" t="s">
+        <v>237</v>
+      </c>
+      <c r="F23" s="34" t="s">
+        <v>238</v>
+      </c>
+      <c r="G23" s="34" t="s">
+        <v>301</v>
+      </c>
+      <c r="H23" s="34" t="s">
+        <v>239</v>
+      </c>
+      <c r="I23" s="33"/>
+      <c r="J23" s="33"/>
+      <c r="K23" s="33"/>
+      <c r="L23" s="33"/>
+      <c r="M23" s="33"/>
+      <c r="N23" s="33"/>
+      <c r="O23" s="33"/>
+    </row>
+    <row r="24" spans="1:15" ht="112" x14ac:dyDescent="0.2">
+      <c r="A24" s="34">
+        <v>26</v>
+      </c>
+      <c r="B24" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" s="34" t="s">
+        <v>240</v>
+      </c>
+      <c r="D24" s="34" t="s">
+        <v>241</v>
+      </c>
+      <c r="E24" s="34" t="s">
+        <v>242</v>
+      </c>
+      <c r="F24" s="34" t="s">
+        <v>243</v>
+      </c>
+      <c r="G24" s="34" t="s">
+        <v>302</v>
+      </c>
+      <c r="H24" s="34" t="s">
+        <v>244</v>
+      </c>
+      <c r="I24" s="33"/>
+      <c r="J24" s="33"/>
+      <c r="K24" s="33"/>
+      <c r="L24" s="33"/>
+      <c r="M24" s="33"/>
+      <c r="N24" s="33"/>
+      <c r="O24" s="33"/>
+    </row>
+    <row r="25" spans="1:15" ht="96" x14ac:dyDescent="0.2">
+      <c r="A25" s="34">
+        <v>27</v>
+      </c>
+      <c r="B25" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" s="34" t="s">
+        <v>245</v>
+      </c>
+      <c r="D25" s="34" t="s">
+        <v>246</v>
+      </c>
+      <c r="E25" s="34" t="s">
+        <v>247</v>
+      </c>
+      <c r="F25" s="34" t="s">
+        <v>248</v>
+      </c>
+      <c r="G25" s="34" t="s">
+        <v>303</v>
+      </c>
+      <c r="H25" s="34" t="s">
+        <v>249</v>
+      </c>
+      <c r="I25" s="33"/>
+      <c r="J25" s="33"/>
+      <c r="K25" s="33"/>
+      <c r="L25" s="33"/>
+      <c r="M25" s="33"/>
+      <c r="N25" s="33"/>
+      <c r="O25" s="33"/>
+    </row>
+    <row r="26" spans="1:15" ht="112" x14ac:dyDescent="0.2">
+      <c r="A26" s="34">
+        <v>28</v>
+      </c>
+      <c r="B26" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="34" t="s">
+        <v>250</v>
+      </c>
+      <c r="D26" s="34" t="s">
+        <v>251</v>
+      </c>
+      <c r="E26" s="34" t="s">
+        <v>252</v>
+      </c>
+      <c r="F26" s="34" t="s">
+        <v>253</v>
+      </c>
+      <c r="G26" s="34" t="s">
+        <v>304</v>
+      </c>
+      <c r="H26" s="34" t="s">
+        <v>254</v>
+      </c>
+      <c r="I26" s="33"/>
+      <c r="J26" s="33"/>
+      <c r="K26" s="33"/>
+      <c r="L26" s="33"/>
+      <c r="M26" s="33"/>
+      <c r="N26" s="33"/>
+      <c r="O26" s="33"/>
+    </row>
+    <row r="27" spans="1:15" ht="112" x14ac:dyDescent="0.2">
+      <c r="A27" s="34">
+        <v>29</v>
+      </c>
+      <c r="B27" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="34" t="s">
+        <v>255</v>
+      </c>
+      <c r="D27" s="34" t="s">
+        <v>256</v>
+      </c>
+      <c r="E27" s="34" t="s">
+        <v>257</v>
+      </c>
+      <c r="F27" s="34" t="s">
+        <v>258</v>
+      </c>
+      <c r="G27" s="34" t="s">
+        <v>305</v>
+      </c>
+      <c r="H27" s="34" t="s">
+        <v>259</v>
+      </c>
+      <c r="I27" s="33"/>
+      <c r="J27" s="33"/>
+      <c r="K27" s="33"/>
+      <c r="L27" s="33"/>
+      <c r="M27" s="33"/>
+      <c r="N27" s="33"/>
+      <c r="O27" s="33"/>
+    </row>
+    <row r="28" spans="1:15" ht="112" x14ac:dyDescent="0.2">
+      <c r="A28" s="34">
+        <v>30</v>
+      </c>
+      <c r="B28" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="34" t="s">
+        <v>260</v>
+      </c>
+      <c r="D28" s="34" t="s">
+        <v>261</v>
+      </c>
+      <c r="E28" s="34" t="s">
+        <v>262</v>
+      </c>
+      <c r="F28" s="34" t="s">
+        <v>263</v>
+      </c>
+      <c r="G28" s="34" t="s">
+        <v>306</v>
+      </c>
+      <c r="H28" s="34" t="s">
+        <v>264</v>
+      </c>
+      <c r="I28" s="33"/>
+      <c r="J28" s="33"/>
+      <c r="K28" s="33"/>
+      <c r="L28" s="33"/>
+      <c r="M28" s="33"/>
+      <c r="N28" s="33"/>
+      <c r="O28" s="33"/>
+    </row>
+    <row r="29" spans="1:15" ht="112" x14ac:dyDescent="0.2">
+      <c r="A29" s="34">
+        <v>31</v>
+      </c>
+      <c r="B29" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="C29" s="34" t="s">
+        <v>265</v>
+      </c>
+      <c r="D29" s="34" t="s">
+        <v>266</v>
+      </c>
+      <c r="E29" s="34" t="s">
+        <v>267</v>
+      </c>
+      <c r="F29" s="34" t="s">
+        <v>268</v>
+      </c>
+      <c r="G29" s="34" t="s">
+        <v>307</v>
+      </c>
+      <c r="H29" s="34" t="s">
+        <v>269</v>
+      </c>
+      <c r="I29" s="33"/>
+      <c r="J29" s="33"/>
+      <c r="K29" s="33"/>
+      <c r="L29" s="33"/>
+      <c r="M29" s="33"/>
+      <c r="N29" s="33"/>
+      <c r="O29" s="33"/>
+    </row>
+    <row r="30" spans="1:15" ht="112" x14ac:dyDescent="0.2">
+      <c r="A30" s="34">
+        <v>32</v>
+      </c>
+      <c r="B30" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="C30" s="34" t="s">
+        <v>270</v>
+      </c>
+      <c r="D30" s="34" t="s">
+        <v>271</v>
+      </c>
+      <c r="E30" s="34" t="s">
+        <v>272</v>
+      </c>
+      <c r="F30" s="34" t="s">
+        <v>314</v>
+      </c>
+      <c r="G30" s="34" t="s">
+        <v>308</v>
+      </c>
+      <c r="H30" s="34" t="s">
+        <v>273</v>
+      </c>
+      <c r="I30" s="33"/>
+      <c r="J30" s="33"/>
+      <c r="K30" s="33"/>
+      <c r="L30" s="33"/>
+      <c r="M30" s="33"/>
+      <c r="N30" s="33"/>
+      <c r="O30" s="33"/>
+    </row>
+    <row r="31" spans="1:15" ht="112" x14ac:dyDescent="0.2">
+      <c r="A31" s="34">
+        <v>33</v>
+      </c>
+      <c r="B31" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="C31" s="34" t="s">
+        <v>274</v>
+      </c>
+      <c r="D31" s="34" t="s">
+        <v>275</v>
+      </c>
+      <c r="E31" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="F31" s="34" t="s">
+        <v>277</v>
+      </c>
+      <c r="G31" s="34" t="s">
+        <v>309</v>
+      </c>
+      <c r="H31" s="34" t="s">
+        <v>278</v>
+      </c>
+      <c r="I31" s="33"/>
+      <c r="J31" s="33"/>
+      <c r="K31" s="33"/>
+      <c r="L31" s="33"/>
+      <c r="M31" s="33"/>
+      <c r="N31" s="33"/>
+      <c r="O31" s="33"/>
+    </row>
+    <row r="32" spans="1:15" ht="128" x14ac:dyDescent="0.2">
+      <c r="A32" s="34">
+        <v>36</v>
+      </c>
+      <c r="B32" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" s="34" t="s">
+        <v>279</v>
+      </c>
+      <c r="D32" s="34" t="s">
+        <v>280</v>
+      </c>
+      <c r="E32" s="34" t="s">
+        <v>281</v>
+      </c>
+      <c r="F32" s="34" t="s">
+        <v>282</v>
+      </c>
+      <c r="G32" s="34" t="s">
+        <v>310</v>
+      </c>
+      <c r="H32" s="34" t="s">
+        <v>283</v>
+      </c>
+      <c r="I32" s="33"/>
+      <c r="J32" s="33"/>
+      <c r="K32" s="33"/>
+      <c r="L32" s="33"/>
+      <c r="M32" s="33"/>
+      <c r="N32" s="33"/>
+      <c r="O32" s="33"/>
+    </row>
+    <row r="33" spans="1:15" ht="128" x14ac:dyDescent="0.2">
+      <c r="A33" s="34">
+        <v>37</v>
+      </c>
+      <c r="B33" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="C33" s="34" t="s">
+        <v>284</v>
+      </c>
+      <c r="D33" s="34" t="s">
+        <v>285</v>
+      </c>
+      <c r="E33" s="34" t="s">
+        <v>286</v>
+      </c>
+      <c r="F33" s="34" t="s">
+        <v>287</v>
+      </c>
+      <c r="G33" s="34" t="s">
+        <v>311</v>
+      </c>
+      <c r="H33" s="34" t="s">
+        <v>288</v>
+      </c>
+      <c r="I33" s="33"/>
+      <c r="J33" s="33"/>
+      <c r="K33" s="33"/>
+      <c r="L33" s="33"/>
+      <c r="M33" s="33"/>
+      <c r="N33" s="33"/>
+      <c r="O33" s="33"/>
+    </row>
+    <row r="34" spans="1:15" ht="128" x14ac:dyDescent="0.2">
+      <c r="A34" s="34">
+        <v>38</v>
+      </c>
+      <c r="B34" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="C34" s="34" t="s">
+        <v>289</v>
+      </c>
+      <c r="D34" s="34" t="s">
+        <v>290</v>
+      </c>
+      <c r="E34" s="34" t="s">
+        <v>291</v>
+      </c>
+      <c r="F34" s="34" t="s">
+        <v>315</v>
+      </c>
+      <c r="G34" s="34" t="s">
+        <v>312</v>
+      </c>
+      <c r="H34" s="34" t="s">
+        <v>292</v>
+      </c>
+      <c r="I34" s="33"/>
+      <c r="J34" s="33"/>
+      <c r="K34" s="33"/>
+      <c r="L34" s="33"/>
+      <c r="M34" s="33"/>
+      <c r="N34" s="33"/>
+      <c r="O34" s="33"/>
+    </row>
+    <row r="35" spans="1:15" ht="128" x14ac:dyDescent="0.2">
+      <c r="A35" s="34">
+        <v>39</v>
+      </c>
+      <c r="B35" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="C35" s="34" t="s">
+        <v>293</v>
+      </c>
+      <c r="D35" s="34" t="s">
+        <v>294</v>
+      </c>
+      <c r="E35" s="34" t="s">
+        <v>295</v>
+      </c>
+      <c r="F35" s="34" t="s">
+        <v>296</v>
+      </c>
+      <c r="G35" s="34" t="s">
+        <v>313</v>
+      </c>
+      <c r="H35" s="34" t="s">
+        <v>297</v>
+      </c>
+      <c r="I35" s="33"/>
+      <c r="J35" s="33"/>
+      <c r="K35" s="33"/>
+      <c r="L35" s="33"/>
+      <c r="M35" s="33"/>
+      <c r="N35" s="33"/>
+      <c r="O35" s="33"/>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A36" s="35"/>
+      <c r="B36" s="36"/>
+      <c r="C36" s="36"/>
+      <c r="D36" s="36"/>
+      <c r="E36" s="36"/>
+      <c r="F36" s="36"/>
+      <c r="G36" s="37"/>
+      <c r="H36" s="36"/>
+      <c r="I36" s="33"/>
+      <c r="J36" s="33"/>
+      <c r="K36" s="33"/>
+      <c r="L36" s="33"/>
+      <c r="M36" s="33"/>
+      <c r="N36" s="33"/>
+      <c r="O36" s="33"/>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A37" s="31"/>
+      <c r="B37" s="32"/>
+      <c r="C37" s="32"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="31"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="33"/>
+      <c r="J37" s="33"/>
+      <c r="K37" s="33"/>
+      <c r="L37" s="33"/>
+      <c r="M37" s="33"/>
+      <c r="N37" s="33"/>
+      <c r="O37" s="33"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A38" s="31"/>
+      <c r="B38" s="32"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="33"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="33"/>
+      <c r="J38" s="33"/>
+      <c r="K38" s="33"/>
+      <c r="L38" s="33"/>
+      <c r="M38" s="33"/>
+      <c r="N38" s="33"/>
+      <c r="O38" s="33"/>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A39" s="31"/>
+      <c r="B39" s="32"/>
+      <c r="C39" s="32"/>
+      <c r="D39" s="32"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="31"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="33"/>
+      <c r="J39" s="33"/>
+      <c r="K39" s="33"/>
+      <c r="L39" s="33"/>
+      <c r="M39" s="33"/>
+      <c r="N39" s="33"/>
+      <c r="O39" s="33"/>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A40" s="31"/>
+      <c r="B40" s="32"/>
+      <c r="C40" s="32"/>
+      <c r="D40" s="32"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="33"/>
+      <c r="H40" s="32"/>
+      <c r="I40" s="33"/>
+      <c r="J40" s="33"/>
+      <c r="K40" s="33"/>
+      <c r="L40" s="33"/>
+      <c r="M40" s="33"/>
+      <c r="N40" s="33"/>
+      <c r="O40" s="33"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A41" s="31"/>
+      <c r="B41" s="32"/>
+      <c r="C41" s="32"/>
+      <c r="D41" s="32"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="31"/>
+      <c r="H41" s="32"/>
+      <c r="I41" s="33"/>
+      <c r="J41" s="33"/>
+      <c r="K41" s="33"/>
+      <c r="L41" s="33"/>
+      <c r="M41" s="33"/>
+      <c r="N41" s="33"/>
+      <c r="O41" s="33"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A42" s="31"/>
+      <c r="B42" s="32"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="32"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="31"/>
+      <c r="H42" s="32"/>
+      <c r="I42" s="33"/>
+      <c r="J42" s="33"/>
+      <c r="K42" s="33"/>
+      <c r="L42" s="33"/>
+      <c r="M42" s="33"/>
+      <c r="N42" s="33"/>
+      <c r="O42" s="33"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A43" s="31"/>
+      <c r="B43" s="32"/>
+      <c r="C43" s="32"/>
+      <c r="D43" s="32"/>
+      <c r="E43" s="32"/>
+      <c r="F43" s="32"/>
+      <c r="G43" s="33"/>
+      <c r="H43" s="32"/>
+      <c r="I43" s="33"/>
+      <c r="J43" s="33"/>
+      <c r="K43" s="33"/>
+      <c r="L43" s="33"/>
+      <c r="M43" s="33"/>
+      <c r="N43" s="33"/>
+      <c r="O43" s="33"/>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A44" s="31"/>
+      <c r="B44" s="32"/>
+      <c r="C44" s="32"/>
+      <c r="D44" s="32"/>
+      <c r="E44" s="32"/>
+      <c r="F44" s="32"/>
+      <c r="G44" s="31"/>
+      <c r="H44" s="32"/>
+      <c r="I44" s="33"/>
+      <c r="J44" s="33"/>
+      <c r="K44" s="33"/>
+      <c r="L44" s="33"/>
+      <c r="M44" s="33"/>
+      <c r="N44" s="33"/>
+      <c r="O44" s="33"/>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A45" s="31"/>
+      <c r="B45" s="32"/>
+      <c r="C45" s="32"/>
+      <c r="D45" s="32"/>
+      <c r="E45" s="32"/>
+      <c r="F45" s="32"/>
+      <c r="G45" s="33"/>
+      <c r="H45" s="32"/>
+      <c r="I45" s="33"/>
+      <c r="J45" s="33"/>
+      <c r="K45" s="33"/>
+      <c r="L45" s="33"/>
+      <c r="M45" s="33"/>
+      <c r="N45" s="33"/>
+      <c r="O45" s="33"/>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A46" s="31"/>
+      <c r="B46" s="32"/>
+      <c r="C46" s="32"/>
+      <c r="D46" s="32"/>
+      <c r="E46" s="32"/>
+      <c r="F46" s="32"/>
+      <c r="G46" s="31"/>
+      <c r="H46" s="32"/>
+      <c r="I46" s="33"/>
+      <c r="J46" s="33"/>
+      <c r="K46" s="33"/>
+      <c r="L46" s="33"/>
+      <c r="M46" s="33"/>
+      <c r="N46" s="33"/>
+      <c r="O46" s="33"/>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A47" s="31"/>
+      <c r="B47" s="32"/>
+      <c r="C47" s="32"/>
+      <c r="D47" s="32"/>
+      <c r="E47" s="32"/>
+      <c r="F47" s="32"/>
+      <c r="G47" s="33"/>
+      <c r="H47" s="32"/>
+      <c r="I47" s="33"/>
+      <c r="J47" s="33"/>
+      <c r="K47" s="33"/>
+      <c r="L47" s="33"/>
+      <c r="M47" s="33"/>
+      <c r="N47" s="33"/>
+      <c r="O47" s="33"/>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A48" s="31"/>
+      <c r="B48" s="32"/>
+      <c r="C48" s="32"/>
+      <c r="D48" s="32"/>
+      <c r="E48" s="32"/>
+      <c r="F48" s="32"/>
+      <c r="G48" s="31"/>
+      <c r="H48" s="32"/>
+      <c r="I48" s="33"/>
+      <c r="J48" s="33"/>
+      <c r="K48" s="33"/>
+      <c r="L48" s="33"/>
+      <c r="M48" s="33"/>
+      <c r="N48" s="33"/>
+      <c r="O48" s="33"/>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A49" s="31"/>
+      <c r="B49" s="32"/>
+      <c r="C49" s="32"/>
+      <c r="D49" s="32"/>
+      <c r="E49" s="32"/>
+      <c r="F49" s="32"/>
+      <c r="G49" s="31"/>
+      <c r="H49" s="32"/>
+      <c r="I49" s="33"/>
+      <c r="J49" s="33"/>
+      <c r="K49" s="33"/>
+      <c r="L49" s="33"/>
+      <c r="M49" s="33"/>
+      <c r="N49" s="33"/>
+      <c r="O49" s="33"/>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A50" s="31"/>
+      <c r="B50" s="32"/>
+      <c r="C50" s="32"/>
+      <c r="D50" s="32"/>
+      <c r="E50" s="32"/>
+      <c r="F50" s="32"/>
+      <c r="G50" s="33"/>
+      <c r="H50" s="32"/>
+      <c r="I50" s="33"/>
+      <c r="J50" s="33"/>
+      <c r="K50" s="33"/>
+      <c r="L50" s="33"/>
+      <c r="M50" s="33"/>
+      <c r="N50" s="33"/>
+      <c r="O50" s="33"/>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A51" s="31"/>
+      <c r="B51" s="32"/>
+      <c r="C51" s="32"/>
+      <c r="D51" s="32"/>
+      <c r="E51" s="32"/>
+      <c r="F51" s="32"/>
+      <c r="G51" s="31"/>
+      <c r="H51" s="32"/>
+      <c r="I51" s="33"/>
+      <c r="J51" s="33"/>
+      <c r="K51" s="33"/>
+      <c r="L51" s="33"/>
+      <c r="M51" s="33"/>
+      <c r="N51" s="33"/>
+      <c r="O51" s="33"/>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A52" s="31"/>
+      <c r="B52" s="32"/>
+      <c r="C52" s="32"/>
+      <c r="D52" s="32"/>
+      <c r="E52" s="32"/>
+      <c r="F52" s="32"/>
+      <c r="G52" s="33"/>
+      <c r="H52" s="32"/>
+      <c r="I52" s="33"/>
+      <c r="J52" s="33"/>
+      <c r="K52" s="33"/>
+      <c r="L52" s="33"/>
+      <c r="M52" s="33"/>
+      <c r="N52" s="33"/>
+      <c r="O52" s="33"/>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A53" s="31"/>
+      <c r="B53" s="32"/>
+      <c r="C53" s="32"/>
+      <c r="D53" s="32"/>
+      <c r="E53" s="32"/>
+      <c r="F53" s="32"/>
+      <c r="G53" s="31"/>
+      <c r="H53" s="32"/>
+      <c r="I53" s="33"/>
+      <c r="J53" s="33"/>
+      <c r="K53" s="33"/>
+      <c r="L53" s="33"/>
+      <c r="M53" s="33"/>
+      <c r="N53" s="33"/>
+      <c r="O53" s="33"/>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A54" s="31"/>
+      <c r="B54" s="32"/>
+      <c r="C54" s="32"/>
+      <c r="D54" s="32"/>
+      <c r="E54" s="32"/>
+      <c r="F54" s="32"/>
+      <c r="G54" s="33"/>
+      <c r="H54" s="32"/>
+      <c r="I54" s="33"/>
+      <c r="J54" s="33"/>
+      <c r="K54" s="33"/>
+      <c r="L54" s="33"/>
+      <c r="M54" s="33"/>
+      <c r="N54" s="33"/>
+      <c r="O54" s="33"/>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A55" s="31"/>
+      <c r="B55" s="32"/>
+      <c r="C55" s="32"/>
+      <c r="D55" s="32"/>
+      <c r="E55" s="32"/>
+      <c r="F55" s="32"/>
+      <c r="G55" s="31"/>
+      <c r="H55" s="32"/>
+      <c r="I55" s="33"/>
+      <c r="J55" s="33"/>
+      <c r="K55" s="33"/>
+      <c r="L55" s="33"/>
+      <c r="M55" s="33"/>
+      <c r="N55" s="33"/>
+      <c r="O55" s="33"/>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A56" s="33"/>
+      <c r="B56" s="33"/>
+      <c r="C56" s="33"/>
+      <c r="D56" s="33"/>
+      <c r="E56" s="33"/>
+      <c r="F56" s="33"/>
+      <c r="G56" s="33"/>
+      <c r="H56" s="33"/>
+      <c r="I56" s="33"/>
+      <c r="J56" s="33"/>
+      <c r="K56" s="33"/>
+      <c r="L56" s="33"/>
+      <c r="M56" s="33"/>
+      <c r="N56" s="33"/>
+      <c r="O56" s="33"/>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A57" s="33"/>
+      <c r="B57" s="33"/>
+      <c r="C57" s="33"/>
+      <c r="D57" s="33"/>
+      <c r="E57" s="33"/>
+      <c r="F57" s="33"/>
+      <c r="G57" s="33"/>
+      <c r="H57" s="33"/>
+      <c r="I57" s="33"/>
+      <c r="J57" s="33"/>
+      <c r="K57" s="33"/>
+      <c r="L57" s="33"/>
+      <c r="M57" s="33"/>
+      <c r="N57" s="33"/>
+      <c r="O57" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1983,24 +3277,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
     </row>
     <row r="3" spans="1:6" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
@@ -2296,20 +3590,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="4" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">

</xml_diff>